<commit_message>
bo sung hinh anh va cap nhat lai tap luat
</commit_message>
<xml_diff>
--- a/data/danh_sach_mon_an.csv.xlsx
+++ b/data/danh_sach_mon_an.csv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BTL TRI TUE NHAN TAO\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9806AD4-A51C-4100-99C8-BF0E72277C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9F2506A-060C-4FDE-8F64-711A1FC9A675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{83411BAF-91DA-4BCB-8993-1CE8A2F2A6CD}"/>
   </bookViews>
@@ -1199,9 +1199,6 @@
     <t>Ngọt, Cay</t>
   </si>
   <si>
-    <t>Thị, Hải sản</t>
-  </si>
-  <si>
     <t>Chua, Ngọt, Béo</t>
   </si>
   <si>
@@ -1260,6 +1257,9 @@
   </si>
   <si>
     <t>Tất cả</t>
+  </si>
+  <si>
+    <t>Bún, Hải sản, Thịt</t>
   </si>
 </sst>
 </file>
@@ -3228,7 +3228,7 @@
         <v>325</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="H31" s="1" t="s">
         <v>345</v>
@@ -3292,7 +3292,7 @@
         <v>325</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>363</v>
+        <v>407</v>
       </c>
       <c r="H33" s="1" t="s">
         <v>349</v>
@@ -3315,7 +3315,7 @@
         <v>16</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>343</v>
+        <v>327</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>21</v>
@@ -3391,7 +3391,7 @@
         <v>122</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>123</v>
@@ -3423,7 +3423,7 @@
         <v>122</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>127</v>
@@ -3472,7 +3472,7 @@
         <v>134</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>23</v>
+        <v>105</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>370</v>
@@ -3487,7 +3487,7 @@
         <v>382</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>349</v>
+        <v>372</v>
       </c>
       <c r="I39" s="1" t="s">
         <v>135</v>
@@ -3583,7 +3583,7 @@
         <v>122</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>149</v>
@@ -3644,7 +3644,7 @@
         <v>336</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>387</v>
+        <v>373</v>
       </c>
       <c r="H44" s="1" t="s">
         <v>322</v>
@@ -3667,7 +3667,7 @@
         <v>23</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>157</v>
@@ -3696,10 +3696,10 @@
         <v>165</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>157</v>
@@ -3708,7 +3708,7 @@
         <v>336</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H46" s="1" t="s">
         <v>322</v>
@@ -3740,10 +3740,10 @@
         <v>325</v>
       </c>
       <c r="G47" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="H47" s="1" t="s">
         <v>391</v>
-      </c>
-      <c r="H47" s="1" t="s">
-        <v>392</v>
       </c>
       <c r="I47" s="1" t="s">
         <v>169</v>
@@ -3775,7 +3775,7 @@
         <v>122</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I48" s="1" t="s">
         <v>173</v>
@@ -3804,7 +3804,7 @@
         <v>325</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="H49" s="1" t="s">
         <v>322</v>
@@ -3856,10 +3856,10 @@
         <v>184</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>139</v>
+        <v>95</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>96</v>
@@ -3868,7 +3868,7 @@
         <v>344</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="H51" s="1" t="s">
         <v>322</v>
@@ -3888,10 +3888,10 @@
         <v>188</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>144</v>
+        <v>82</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>96</v>
@@ -3900,7 +3900,7 @@
         <v>336</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H52" s="1" t="s">
         <v>322</v>
@@ -3955,7 +3955,7 @@
         <v>144</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>96</v>
@@ -3993,7 +3993,7 @@
         <v>38</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>377</v>
@@ -4028,7 +4028,7 @@
         <v>354</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="H56" s="1" t="s">
         <v>345</v>
@@ -4063,7 +4063,7 @@
         <v>122</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I57" s="1" t="s">
         <v>209</v>
@@ -4115,7 +4115,7 @@
         <v>144</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>38</v>
@@ -4176,10 +4176,10 @@
         <v>223</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>144</v>
+        <v>16</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>224</v>
@@ -4287,7 +4287,7 @@
         <v>122</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I64" s="1" t="s">
         <v>238</v>
@@ -4339,7 +4339,7 @@
         <v>144</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>48</v>
@@ -4371,7 +4371,7 @@
         <v>23</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>48</v>
@@ -4380,7 +4380,7 @@
         <v>344</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H67" s="1" t="s">
         <v>322</v>
@@ -4499,7 +4499,7 @@
         <v>144</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>21</v>
@@ -4540,7 +4540,7 @@
         <v>293</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="H72" s="1" t="s">
         <v>349</v>
@@ -4569,7 +4569,7 @@
         <v>33</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G73" s="8" t="s">
         <v>369</v>

</xml_diff>

<commit_message>
cap nhat mon an thieu thong tin
</commit_message>
<xml_diff>
--- a/data/danh_sach_mon_an.csv.xlsx
+++ b/data/danh_sach_mon_an.csv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BTL TRI TUE NHAN TAO\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9F2506A-060C-4FDE-8F64-711A1FC9A675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{99CEDDF4-EBB7-4EA4-AF8B-3FA77AA85051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{83411BAF-91DA-4BCB-8993-1CE8A2F2A6CD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="409">
   <si>
     <t>id</t>
   </si>
@@ -1260,6 +1260,9 @@
   </si>
   <si>
     <t>Bún, Hải sản, Thịt</t>
+  </si>
+  <si>
+    <t>Món cháo, Món lẩu</t>
   </si>
 </sst>
 </file>
@@ -3248,7 +3251,7 @@
         <v>104</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>105</v>
+        <v>408</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>343</v>

</xml_diff>